<commit_message>
Auto update RUP 2026-07-07 10:44:59
</commit_message>
<xml_diff>
--- a/output/rup/2024/Rekap RUP Tahun 2024 (2026-07-07).xlsx
+++ b/output/rup/2024/Rekap RUP Tahun 2024 (2026-07-07).xlsx
@@ -437,17 +437,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,25 +471,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Paket Penyedia</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>RUP Penyedia</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Paket Swakelola</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>RUP Swakelola</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Total Paket Terumumkan</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Total RUP Terumumkan</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Selisih RUP Terumumkan</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Persentase</t>
         </is>
@@ -505,18 +523,27 @@
         <v>6609077174</v>
       </c>
       <c r="D2" s="3" t="n">
+        <v>106</v>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>1733202792</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="F2" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>5444982208</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="H2" s="3" t="n">
+        <v>163</v>
+      </c>
+      <c r="I2" s="3" t="n">
         <v>7178185000</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>569107826</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>108.6110028831084</v>
       </c>
     </row>
@@ -533,18 +560,27 @@
         <v>6012052325</v>
       </c>
       <c r="D3" s="3" t="n">
+        <v>131</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>2653333445</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="F3" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>3358718880</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="H3" s="3" t="n">
+        <v>194</v>
+      </c>
+      <c r="I3" s="3" t="n">
         <v>6012052325</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="n">
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
         <v>100</v>
       </c>
     </row>
@@ -561,18 +597,27 @@
         <v>9791467550</v>
       </c>
       <c r="D4" s="3" t="n">
+        <v>124</v>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>5618515110</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="F4" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>4172952440</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="H4" s="3" t="n">
+        <v>222</v>
+      </c>
+      <c r="I4" s="3" t="n">
         <v>9791467550</v>
       </c>
-      <c r="G4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="n">
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
         <v>100</v>
       </c>
     </row>
@@ -589,18 +634,27 @@
         <v>4030513379</v>
       </c>
       <c r="D5" s="3" t="n">
+        <v>127</v>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>2113075839</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="F5" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>2196598687</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="H5" s="3" t="n">
+        <v>181</v>
+      </c>
+      <c r="I5" s="3" t="n">
         <v>4309674526</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="J5" s="3" t="n">
         <v>279161147</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>106.9261932848183</v>
       </c>
     </row>
@@ -617,18 +671,27 @@
         <v>11462609088</v>
       </c>
       <c r="D6" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>6683247723</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="F6" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>4779361365</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="H6" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="I6" s="3" t="n">
         <v>11462609088</v>
       </c>
-      <c r="G6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="n">
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
         <v>100</v>
       </c>
     </row>
@@ -645,18 +708,27 @@
         <v>10636003247</v>
       </c>
       <c r="D7" s="3" t="n">
+        <v>140</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>6968017137</v>
       </c>
-      <c r="E7" s="3" t="n">
+      <c r="F7" s="3" t="n">
+        <v>103</v>
+      </c>
+      <c r="G7" s="3" t="n">
         <v>4927122922</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="H7" s="3" t="n">
+        <v>243</v>
+      </c>
+      <c r="I7" s="3" t="n">
         <v>11895140059</v>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="J7" s="3" t="n">
         <v>1259136812</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>111.838439522432</v>
       </c>
     </row>
@@ -684,7 +756,16 @@
       <c r="G8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -712,7 +793,16 @@
       <c r="G9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -729,18 +819,27 @@
         <v>9945535255</v>
       </c>
       <c r="D10" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="E10" s="3" t="n">
         <v>8982974966</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="F10" s="3" t="n">
+        <v>78</v>
+      </c>
+      <c r="G10" s="3" t="n">
         <v>4610675900</v>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="H10" s="3" t="n">
+        <v>346</v>
+      </c>
+      <c r="I10" s="3" t="n">
         <v>13593650866</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="J10" s="3" t="n">
         <v>3648115611</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>136.6809379029244</v>
       </c>
     </row>
@@ -757,18 +856,27 @@
         <v>2132532692</v>
       </c>
       <c r="D11" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="E11" s="3" t="n">
         <v>2028695337</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="F11" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>996519388</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="H11" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="I11" s="3" t="n">
         <v>3025214725</v>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="J11" s="3" t="n">
         <v>892682033</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>141.86018044876</v>
       </c>
     </row>
@@ -785,18 +893,27 @@
         <v>55370742582</v>
       </c>
       <c r="D12" s="3" t="n">
+        <v>458</v>
+      </c>
+      <c r="E12" s="3" t="n">
         <v>34635674396</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="F12" s="3" t="n">
+        <v>329</v>
+      </c>
+      <c r="G12" s="3" t="n">
         <v>52892549642</v>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="H12" s="3" t="n">
+        <v>787</v>
+      </c>
+      <c r="I12" s="3" t="n">
         <v>87528224038</v>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="J12" s="3" t="n">
         <v>32157481456</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>158.0766664062291</v>
       </c>
     </row>
@@ -813,18 +930,27 @@
         <v>12842405000</v>
       </c>
       <c r="D13" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="E13" s="3" t="n">
         <v>6326236088</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="F13" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G13" s="3" t="n">
         <v>1243826820</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="H13" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="I13" s="3" t="n">
         <v>7570062908</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="J13" s="3" t="n">
         <v>-5272342092</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>58.94583536339183</v>
       </c>
     </row>
@@ -841,18 +967,27 @@
         <v>20127505472</v>
       </c>
       <c r="D14" s="3" t="n">
+        <v>146</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>11189831295</v>
       </c>
-      <c r="E14" s="3" t="n">
+      <c r="F14" s="3" t="n">
+        <v>78</v>
+      </c>
+      <c r="G14" s="3" t="n">
         <v>13435144705</v>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="H14" s="3" t="n">
+        <v>224</v>
+      </c>
+      <c r="I14" s="3" t="n">
         <v>24624976000</v>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="J14" s="3" t="n">
         <v>4497470528</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>122.3448978029422</v>
       </c>
     </row>
@@ -869,18 +1004,27 @@
         <v>5386064763</v>
       </c>
       <c r="D15" s="3" t="n">
+        <v>331</v>
+      </c>
+      <c r="E15" s="3" t="n">
         <v>9964807080</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="F15" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="G15" s="3" t="n">
         <v>2268633919</v>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="H15" s="3" t="n">
+        <v>420</v>
+      </c>
+      <c r="I15" s="3" t="n">
         <v>12233440999</v>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="J15" s="3" t="n">
         <v>6847376236</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>227.1313386916287</v>
       </c>
     </row>
@@ -897,18 +1041,27 @@
         <v>39609960852</v>
       </c>
       <c r="D16" s="3" t="n">
+        <v>1095</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>317994180779</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="F16" s="3" t="n">
+        <v>422</v>
+      </c>
+      <c r="G16" s="3" t="n">
         <v>9258828108</v>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="H16" s="3" t="n">
+        <v>1517</v>
+      </c>
+      <c r="I16" s="3" t="n">
         <v>327253008887</v>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="J16" s="3" t="n">
         <v>287643048035</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>826.1886703442077</v>
       </c>
     </row>
@@ -925,18 +1078,27 @@
         <v>2425631177</v>
       </c>
       <c r="D17" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>2960870051</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="F17" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G17" s="3" t="n">
         <v>1575658630</v>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="H17" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="I17" s="3" t="n">
         <v>4536528681</v>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="J17" s="3" t="n">
         <v>2110897504</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>187.0246690434916</v>
       </c>
     </row>
@@ -953,18 +1115,27 @@
         <v>4580673342</v>
       </c>
       <c r="D18" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="E18" s="3" t="n">
         <v>849571490</v>
       </c>
-      <c r="E18" s="3" t="n">
+      <c r="F18" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="G18" s="3" t="n">
         <v>3765014884</v>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="H18" s="3" t="n">
+        <v>167</v>
+      </c>
+      <c r="I18" s="3" t="n">
         <v>4614586374</v>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="J18" s="3" t="n">
         <v>33913032</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>100.7403503692143</v>
       </c>
     </row>
@@ -981,18 +1152,27 @@
         <v>7304364300</v>
       </c>
       <c r="D19" s="3" t="n">
+        <v>214</v>
+      </c>
+      <c r="E19" s="3" t="n">
         <v>6751113361</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="F19" s="3" t="n">
+        <v>125</v>
+      </c>
+      <c r="G19" s="3" t="n">
         <v>4585716639</v>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="H19" s="3" t="n">
+        <v>339</v>
+      </c>
+      <c r="I19" s="3" t="n">
         <v>11336830000</v>
       </c>
-      <c r="G19" s="3" t="n">
+      <c r="J19" s="3" t="n">
         <v>4032465700</v>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="K19" s="4" t="n">
         <v>155.2062511449491</v>
       </c>
     </row>
@@ -1009,18 +1189,27 @@
         <v>11122551000</v>
       </c>
       <c r="D20" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>4681921860</v>
       </c>
-      <c r="E20" s="3" t="n">
+      <c r="F20" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G20" s="3" t="n">
         <v>474241098</v>
       </c>
-      <c r="F20" s="3" t="n">
+      <c r="H20" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="I20" s="3" t="n">
         <v>5156162958</v>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="J20" s="3" t="n">
         <v>-5966388042</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>46.35773715939806</v>
       </c>
     </row>
@@ -1037,18 +1226,27 @@
         <v>43445822859</v>
       </c>
       <c r="D21" s="3" t="n">
+        <v>584</v>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>35520107125</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="F21" s="3" t="n">
+        <v>227</v>
+      </c>
+      <c r="G21" s="3" t="n">
         <v>69692221050</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="H21" s="3" t="n">
+        <v>811</v>
+      </c>
+      <c r="I21" s="3" t="n">
         <v>105212328175</v>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="J21" s="3" t="n">
         <v>61766505316</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>242.169030878891</v>
       </c>
     </row>
@@ -1065,18 +1263,27 @@
         <v>12137177249</v>
       </c>
       <c r="D22" s="3" t="n">
+        <v>158</v>
+      </c>
+      <c r="E22" s="3" t="n">
         <v>11796946046</v>
       </c>
-      <c r="E22" s="3" t="n">
+      <c r="F22" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="G22" s="3" t="n">
         <v>3348905644</v>
       </c>
-      <c r="F22" s="3" t="n">
+      <c r="H22" s="3" t="n">
+        <v>247</v>
+      </c>
+      <c r="I22" s="3" t="n">
         <v>15145851690</v>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="J22" s="3" t="n">
         <v>3008674441</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>124.7889140883057</v>
       </c>
     </row>
@@ -1093,18 +1300,27 @@
         <v>12552736040</v>
       </c>
       <c r="D23" s="3" t="n">
+        <v>204</v>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>15907298949</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="F23" s="3" t="n">
+        <v>128</v>
+      </c>
+      <c r="G23" s="3" t="n">
         <v>2649508725</v>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="H23" s="3" t="n">
+        <v>332</v>
+      </c>
+      <c r="I23" s="3" t="n">
         <v>18556807674</v>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="J23" s="3" t="n">
         <v>6004071634</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="K23" s="4" t="n">
         <v>147.8307805953036</v>
       </c>
     </row>
@@ -1121,18 +1337,27 @@
         <v>10762794932</v>
       </c>
       <c r="D24" s="3" t="n">
+        <v>148</v>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>6278519204</v>
       </c>
-      <c r="E24" s="3" t="n">
+      <c r="F24" s="3" t="n">
+        <v>102</v>
+      </c>
+      <c r="G24" s="3" t="n">
         <v>5652777032</v>
       </c>
-      <c r="F24" s="3" t="n">
+      <c r="H24" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="I24" s="3" t="n">
         <v>11931296236</v>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="J24" s="3" t="n">
         <v>1168501304</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>110.8568574555463</v>
       </c>
     </row>
@@ -1149,18 +1374,27 @@
         <v>2098105819</v>
       </c>
       <c r="D25" s="3" t="n">
+        <v>144</v>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>1859979870</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="F25" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G25" s="3" t="n">
         <v>1407337188</v>
       </c>
-      <c r="F25" s="3" t="n">
+      <c r="H25" s="3" t="n">
+        <v>193</v>
+      </c>
+      <c r="I25" s="3" t="n">
         <v>3267317058</v>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="J25" s="3" t="n">
         <v>1169211239</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="K25" s="4" t="n">
         <v>155.7269909082693</v>
       </c>
     </row>
@@ -1177,18 +1411,27 @@
         <v>14825840621</v>
       </c>
       <c r="D26" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>22831397905</v>
       </c>
-      <c r="E26" s="3" t="n">
+      <c r="F26" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="G26" s="3" t="n">
         <v>7666073095</v>
       </c>
-      <c r="F26" s="3" t="n">
+      <c r="H26" s="3" t="n">
+        <v>309</v>
+      </c>
+      <c r="I26" s="3" t="n">
         <v>30497471000</v>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="J26" s="3" t="n">
         <v>15671630379</v>
       </c>
-      <c r="H26" s="4" t="n">
+      <c r="K26" s="4" t="n">
         <v>205.7048350890942</v>
       </c>
     </row>
@@ -1205,18 +1448,27 @@
         <v>3267923856</v>
       </c>
       <c r="D27" s="3" t="n">
+        <v>282</v>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>26567359952</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="F27" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="G27" s="3" t="n">
         <v>3213603117</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="H27" s="3" t="n">
+        <v>346</v>
+      </c>
+      <c r="I27" s="3" t="n">
         <v>29780963069</v>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="J27" s="3" t="n">
         <v>26513039213</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>911.3114130343433</v>
       </c>
     </row>
@@ -1233,18 +1485,27 @@
         <v>4567996790</v>
       </c>
       <c r="D28" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="E28" s="3" t="n">
         <v>3837345154</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="F28" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="G28" s="3" t="n">
         <v>2932950220</v>
       </c>
-      <c r="F28" s="3" t="n">
+      <c r="H28" s="3" t="n">
+        <v>218</v>
+      </c>
+      <c r="I28" s="3" t="n">
         <v>6770295374</v>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="J28" s="3" t="n">
         <v>2202298584</v>
       </c>
-      <c r="H28" s="4" t="n">
+      <c r="K28" s="4" t="n">
         <v>148.2114739839824</v>
       </c>
     </row>
@@ -1261,18 +1522,27 @@
         <v>4933959703</v>
       </c>
       <c r="D29" s="3" t="n">
+        <v>174</v>
+      </c>
+      <c r="E29" s="3" t="n">
         <v>3645691634</v>
       </c>
-      <c r="E29" s="3" t="n">
+      <c r="F29" s="3" t="n">
+        <v>104</v>
+      </c>
+      <c r="G29" s="3" t="n">
         <v>3623037902</v>
       </c>
-      <c r="F29" s="3" t="n">
+      <c r="H29" s="3" t="n">
+        <v>278</v>
+      </c>
+      <c r="I29" s="3" t="n">
         <v>7268729536</v>
       </c>
-      <c r="G29" s="3" t="n">
+      <c r="J29" s="3" t="n">
         <v>2334769833</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="K29" s="4" t="n">
         <v>147.320407411929</v>
       </c>
     </row>
@@ -1289,18 +1559,27 @@
         <v>9237813308</v>
       </c>
       <c r="D30" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="E30" s="3" t="n">
         <v>3377043035</v>
       </c>
-      <c r="E30" s="3" t="n">
+      <c r="F30" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G30" s="3" t="n">
         <v>7483476980</v>
       </c>
-      <c r="F30" s="3" t="n">
+      <c r="H30" s="3" t="n">
+        <v>129</v>
+      </c>
+      <c r="I30" s="3" t="n">
         <v>10860520015</v>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="J30" s="3" t="n">
         <v>1622706707</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="K30" s="4" t="n">
         <v>117.5659179602031</v>
       </c>
     </row>
@@ -1328,7 +1607,16 @@
       <c r="G31" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H31" s="4" t="n">
+      <c r="H31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1345,18 +1633,27 @@
         <v>5738046854</v>
       </c>
       <c r="D32" s="3" t="n">
+        <v>318</v>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>5992729771</v>
       </c>
-      <c r="E32" s="3" t="n">
+      <c r="F32" s="3" t="n">
+        <v>204</v>
+      </c>
+      <c r="G32" s="3" t="n">
         <v>3813448947</v>
       </c>
-      <c r="F32" s="3" t="n">
+      <c r="H32" s="3" t="n">
+        <v>522</v>
+      </c>
+      <c r="I32" s="3" t="n">
         <v>9806178718</v>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="J32" s="3" t="n">
         <v>4068131864</v>
       </c>
-      <c r="H32" s="4" t="n">
+      <c r="K32" s="4" t="n">
         <v>170.8975016675596</v>
       </c>
     </row>
@@ -1373,18 +1670,27 @@
         <v>1394256396</v>
       </c>
       <c r="D33" s="3" t="n">
+        <v>81</v>
+      </c>
+      <c r="E33" s="3" t="n">
         <v>1007256017</v>
       </c>
-      <c r="E33" s="3" t="n">
+      <c r="F33" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="G33" s="3" t="n">
         <v>1001904150</v>
       </c>
-      <c r="F33" s="3" t="n">
+      <c r="H33" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="I33" s="3" t="n">
         <v>2009160167</v>
       </c>
-      <c r="G33" s="3" t="n">
+      <c r="J33" s="3" t="n">
         <v>614903771</v>
       </c>
-      <c r="H33" s="4" t="n">
+      <c r="K33" s="4" t="n">
         <v>144.1026322535873</v>
       </c>
     </row>
@@ -1401,18 +1707,27 @@
         <v>2191867550</v>
       </c>
       <c r="D34" s="3" t="n">
+        <v>103</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>1814789781</v>
       </c>
-      <c r="E34" s="3" t="n">
+      <c r="F34" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="G34" s="3" t="n">
         <v>1606688219</v>
       </c>
-      <c r="F34" s="3" t="n">
+      <c r="H34" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="I34" s="3" t="n">
         <v>3421478000</v>
       </c>
-      <c r="G34" s="3" t="n">
+      <c r="J34" s="3" t="n">
         <v>1229610450</v>
       </c>
-      <c r="H34" s="4" t="n">
+      <c r="K34" s="4" t="n">
         <v>156.0987569709675</v>
       </c>
     </row>
@@ -1429,18 +1744,27 @@
         <v>2844298123</v>
       </c>
       <c r="D35" s="3" t="n">
+        <v>159</v>
+      </c>
+      <c r="E35" s="3" t="n">
         <v>3309363185</v>
       </c>
-      <c r="E35" s="3" t="n">
+      <c r="F35" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="G35" s="3" t="n">
         <v>1531021815</v>
       </c>
-      <c r="F35" s="3" t="n">
+      <c r="H35" s="3" t="n">
+        <v>231</v>
+      </c>
+      <c r="I35" s="3" t="n">
         <v>4840385000</v>
       </c>
-      <c r="G35" s="3" t="n">
+      <c r="J35" s="3" t="n">
         <v>1996086877</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="K35" s="4" t="n">
         <v>170.1785393330937</v>
       </c>
     </row>
@@ -1457,18 +1781,27 @@
         <v>791403947</v>
       </c>
       <c r="D36" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="E36" s="3" t="n">
         <v>890889831</v>
       </c>
-      <c r="E36" s="3" t="n">
+      <c r="F36" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G36" s="3" t="n">
         <v>500038380</v>
       </c>
-      <c r="F36" s="3" t="n">
+      <c r="H36" s="3" t="n">
+        <v>105</v>
+      </c>
+      <c r="I36" s="3" t="n">
         <v>1390928211</v>
       </c>
-      <c r="G36" s="3" t="n">
+      <c r="J36" s="3" t="n">
         <v>599524264</v>
       </c>
-      <c r="H36" s="4" t="n">
+      <c r="K36" s="4" t="n">
         <v>175.754520339788</v>
       </c>
     </row>
@@ -1485,18 +1818,27 @@
         <v>631195426</v>
       </c>
       <c r="D37" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="E37" s="3" t="n">
         <v>759360980</v>
       </c>
-      <c r="E37" s="3" t="n">
+      <c r="F37" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="G37" s="3" t="n">
         <v>408872020</v>
       </c>
-      <c r="F37" s="3" t="n">
+      <c r="H37" s="3" t="n">
+        <v>156</v>
+      </c>
+      <c r="I37" s="3" t="n">
         <v>1168233000</v>
       </c>
-      <c r="G37" s="3" t="n">
+      <c r="J37" s="3" t="n">
         <v>537037574</v>
       </c>
-      <c r="H37" s="4" t="n">
+      <c r="K37" s="4" t="n">
         <v>185.0826149681256</v>
       </c>
     </row>
@@ -1524,7 +1866,16 @@
       <c r="G38" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="4" t="n">
+      <c r="H38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1552,7 +1903,16 @@
       <c r="G39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H39" s="4" t="n">
+      <c r="H39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1580,7 +1940,16 @@
       <c r="G40" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H40" s="4" t="n">
+      <c r="H40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1608,7 +1977,16 @@
       <c r="G41" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="4" t="n">
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1636,7 +2014,16 @@
       <c r="G42" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H42" s="4" t="n">
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1664,7 +2051,16 @@
       <c r="G43" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H43" s="4" t="n">
+      <c r="H43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1692,7 +2088,16 @@
       <c r="G44" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H44" s="4" t="n">
+      <c r="H44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1720,7 +2125,16 @@
       <c r="G45" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H45" s="4" t="n">
+      <c r="H45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1748,7 +2162,16 @@
       <c r="G46" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H46" s="4" t="n">
+      <c r="H46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1776,7 +2199,16 @@
       <c r="G47" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H47" s="4" t="n">
+      <c r="H47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1804,7 +2236,16 @@
       <c r="G48" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H48" s="4" t="n">
+      <c r="H48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1832,7 +2273,16 @@
       <c r="G49" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H49" s="4" t="n">
+      <c r="H49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1860,7 +2310,16 @@
       <c r="G50" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H50" s="4" t="n">
+      <c r="H50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1888,7 +2347,16 @@
       <c r="G51" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H51" s="4" t="n">
+      <c r="H51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1916,7 +2384,16 @@
       <c r="G52" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H52" s="4" t="n">
+      <c r="H52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1944,7 +2421,16 @@
       <c r="G53" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H53" s="4" t="n">
+      <c r="H53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1972,7 +2458,16 @@
       <c r="G54" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H54" s="4" t="n">
+      <c r="H54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2000,7 +2495,16 @@
       <c r="G55" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H55" s="4" t="n">
+      <c r="H55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2028,7 +2532,16 @@
       <c r="G56" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H56" s="4" t="n">
+      <c r="H56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2045,18 +2558,27 @@
         <v>1475675849</v>
       </c>
       <c r="D57" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="E57" s="3" t="n">
         <v>745060149</v>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="F57" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G57" s="3" t="n">
         <v>786198000</v>
       </c>
-      <c r="F57" s="3" t="n">
+      <c r="H57" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I57" s="3" t="n">
         <v>1531258149</v>
       </c>
-      <c r="G57" s="3" t="n">
+      <c r="J57" s="3" t="n">
         <v>55582300</v>
       </c>
-      <c r="H57" s="4" t="n">
+      <c r="K57" s="4" t="n">
         <v>103.7665656748171</v>
       </c>
     </row>
@@ -2073,18 +2595,27 @@
         <v>1379727201</v>
       </c>
       <c r="D58" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E58" s="3" t="n">
         <v>440906073</v>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="F58" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G58" s="3" t="n">
         <v>908590848</v>
       </c>
-      <c r="F58" s="3" t="n">
+      <c r="H58" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="I58" s="3" t="n">
         <v>1349496921</v>
       </c>
-      <c r="G58" s="3" t="n">
+      <c r="J58" s="3" t="n">
         <v>-30230280</v>
       </c>
-      <c r="H58" s="4" t="n">
+      <c r="K58" s="4" t="n">
         <v>97.80896687561935</v>
       </c>
     </row>
@@ -2101,18 +2632,27 @@
         <v>1194175835</v>
       </c>
       <c r="D59" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="E59" s="3" t="n">
         <v>178478188</v>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="F59" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="G59" s="3" t="n">
         <v>787487417</v>
       </c>
-      <c r="F59" s="3" t="n">
+      <c r="H59" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="I59" s="3" t="n">
         <v>965965605</v>
       </c>
-      <c r="G59" s="3" t="n">
+      <c r="J59" s="3" t="n">
         <v>-228210230</v>
       </c>
-      <c r="H59" s="4" t="n">
+      <c r="K59" s="4" t="n">
         <v>80.889729693785</v>
       </c>
     </row>
@@ -2129,18 +2669,27 @@
         <v>1539482505</v>
       </c>
       <c r="D60" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="E60" s="3" t="n">
         <v>624864225</v>
       </c>
-      <c r="E60" s="3" t="n">
+      <c r="F60" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G60" s="3" t="n">
         <v>269990000</v>
       </c>
-      <c r="F60" s="3" t="n">
+      <c r="H60" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="I60" s="3" t="n">
         <v>894854225</v>
       </c>
-      <c r="G60" s="3" t="n">
+      <c r="J60" s="3" t="n">
         <v>-644628280</v>
       </c>
-      <c r="H60" s="4" t="n">
+      <c r="K60" s="4" t="n">
         <v>58.12694993893419</v>
       </c>
     </row>
@@ -2157,18 +2706,27 @@
         <v>1389901000</v>
       </c>
       <c r="D61" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E61" s="3" t="n">
         <v>441476300</v>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="F61" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="G61" s="3" t="n">
         <v>922593600</v>
       </c>
-      <c r="F61" s="3" t="n">
+      <c r="H61" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="I61" s="3" t="n">
         <v>1364069900</v>
       </c>
-      <c r="G61" s="3" t="n">
+      <c r="J61" s="3" t="n">
         <v>-25831100</v>
       </c>
-      <c r="H61" s="4" t="n">
+      <c r="K61" s="4" t="n">
         <v>98.14151511510532</v>
       </c>
     </row>
@@ -2185,18 +2743,27 @@
         <v>2096260926</v>
       </c>
       <c r="D62" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="E62" s="3" t="n">
         <v>955140035</v>
       </c>
-      <c r="E62" s="3" t="n">
+      <c r="F62" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G62" s="3" t="n">
         <v>1120490689</v>
       </c>
-      <c r="F62" s="3" t="n">
+      <c r="H62" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="I62" s="3" t="n">
         <v>2075630724</v>
       </c>
-      <c r="G62" s="3" t="n">
+      <c r="J62" s="3" t="n">
         <v>-20630202</v>
       </c>
-      <c r="H62" s="4" t="n">
+      <c r="K62" s="4" t="n">
         <v>99.0158571509814</v>
       </c>
     </row>
@@ -2213,18 +2780,27 @@
         <v>1202086101</v>
       </c>
       <c r="D63" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E63" s="3" t="n">
         <v>440325167</v>
       </c>
-      <c r="E63" s="3" t="n">
+      <c r="F63" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G63" s="3" t="n">
         <v>742215917</v>
       </c>
-      <c r="F63" s="3" t="n">
+      <c r="H63" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="I63" s="3" t="n">
         <v>1182541084</v>
       </c>
-      <c r="G63" s="3" t="n">
+      <c r="J63" s="3" t="n">
         <v>-19545017</v>
       </c>
-      <c r="H63" s="4" t="n">
+      <c r="K63" s="4" t="n">
         <v>98.3740751195991</v>
       </c>
     </row>
@@ -2241,18 +2817,27 @@
         <v>1583413174</v>
       </c>
       <c r="D64" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E64" s="3" t="n">
         <v>706442561</v>
       </c>
-      <c r="E64" s="3" t="n">
+      <c r="F64" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G64" s="3" t="n">
         <v>940532909</v>
       </c>
-      <c r="F64" s="3" t="n">
+      <c r="H64" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="I64" s="3" t="n">
         <v>1646975470</v>
       </c>
-      <c r="G64" s="3" t="n">
+      <c r="J64" s="3" t="n">
         <v>63562296</v>
       </c>
-      <c r="H64" s="4" t="n">
+      <c r="K64" s="4" t="n">
         <v>104.0142583782747</v>
       </c>
     </row>
@@ -2269,18 +2854,27 @@
         <v>1460797490</v>
       </c>
       <c r="D65" s="3" t="n">
+        <v>190</v>
+      </c>
+      <c r="E65" s="3" t="n">
         <v>761668070</v>
       </c>
-      <c r="E65" s="3" t="n">
+      <c r="F65" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="G65" s="3" t="n">
         <v>762155799</v>
       </c>
-      <c r="F65" s="3" t="n">
+      <c r="H65" s="3" t="n">
+        <v>275</v>
+      </c>
+      <c r="I65" s="3" t="n">
         <v>1523823869</v>
       </c>
-      <c r="G65" s="3" t="n">
+      <c r="J65" s="3" t="n">
         <v>63026379</v>
       </c>
-      <c r="H65" s="4" t="n">
+      <c r="K65" s="4" t="n">
         <v>104.3145185716331</v>
       </c>
     </row>
@@ -2297,18 +2891,27 @@
         <v>1463104211</v>
       </c>
       <c r="D66" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="E66" s="3" t="n">
         <v>631541279</v>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="F66" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G66" s="3" t="n">
         <v>284070000</v>
       </c>
-      <c r="F66" s="3" t="n">
+      <c r="H66" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="I66" s="3" t="n">
         <v>915611279</v>
       </c>
-      <c r="G66" s="3" t="n">
+      <c r="J66" s="3" t="n">
         <v>-547492932</v>
       </c>
-      <c r="H66" s="4" t="n">
+      <c r="K66" s="4" t="n">
         <v>62.58004536629688</v>
       </c>
     </row>
@@ -2325,18 +2928,27 @@
         <v>1382930759</v>
       </c>
       <c r="D67" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E67" s="3" t="n">
         <v>568783735</v>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="F67" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G67" s="3" t="n">
         <v>888121939</v>
       </c>
-      <c r="F67" s="3" t="n">
+      <c r="H67" s="3" t="n">
+        <v>66</v>
+      </c>
+      <c r="I67" s="3" t="n">
         <v>1456905674</v>
       </c>
-      <c r="G67" s="3" t="n">
+      <c r="J67" s="3" t="n">
         <v>73974915</v>
       </c>
-      <c r="H67" s="4" t="n">
+      <c r="K67" s="4" t="n">
         <v>105.3491409109659</v>
       </c>
     </row>
@@ -2353,18 +2965,27 @@
         <v>1290067087</v>
       </c>
       <c r="D68" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E68" s="3" t="n">
         <v>362094886</v>
       </c>
-      <c r="E68" s="3" t="n">
+      <c r="F68" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G68" s="3" t="n">
         <v>930808462</v>
       </c>
-      <c r="F68" s="3" t="n">
+      <c r="H68" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="I68" s="3" t="n">
         <v>1292903348</v>
       </c>
-      <c r="G68" s="3" t="n">
+      <c r="J68" s="3" t="n">
         <v>2836261</v>
       </c>
-      <c r="H68" s="4" t="n">
+      <c r="K68" s="4" t="n">
         <v>100.2198537602099</v>
       </c>
     </row>
@@ -2381,18 +3002,27 @@
         <v>1210534592</v>
       </c>
       <c r="D69" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E69" s="3" t="n">
         <v>356477825</v>
       </c>
-      <c r="E69" s="3" t="n">
+      <c r="F69" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G69" s="3" t="n">
         <v>854056767</v>
       </c>
-      <c r="F69" s="3" t="n">
+      <c r="H69" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I69" s="3" t="n">
         <v>1210534592</v>
       </c>
-      <c r="G69" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H69" s="4" t="n">
+      <c r="J69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="4" t="n">
         <v>100</v>
       </c>
     </row>
@@ -2409,18 +3039,27 @@
         <v>1310845327</v>
       </c>
       <c r="D70" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E70" s="3" t="n">
         <v>408906730</v>
       </c>
-      <c r="E70" s="3" t="n">
+      <c r="F70" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="G70" s="3" t="n">
         <v>904292417</v>
       </c>
-      <c r="F70" s="3" t="n">
+      <c r="H70" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="I70" s="3" t="n">
         <v>1313199147</v>
       </c>
-      <c r="G70" s="3" t="n">
+      <c r="J70" s="3" t="n">
         <v>2353820</v>
       </c>
-      <c r="H70" s="4" t="n">
+      <c r="K70" s="4" t="n">
         <v>100.1795650449002</v>
       </c>
     </row>
@@ -2437,18 +3076,27 @@
         <v>1223060009</v>
       </c>
       <c r="D71" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="E71" s="3" t="n">
         <v>272362442</v>
       </c>
-      <c r="E71" s="3" t="n">
+      <c r="F71" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G71" s="3" t="n">
         <v>815205667</v>
       </c>
-      <c r="F71" s="3" t="n">
+      <c r="H71" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="I71" s="3" t="n">
         <v>1087568109</v>
       </c>
-      <c r="G71" s="3" t="n">
+      <c r="J71" s="3" t="n">
         <v>-135491900</v>
       </c>
-      <c r="H71" s="4" t="n">
+      <c r="K71" s="4" t="n">
         <v>88.92189271148018</v>
       </c>
     </row>
@@ -2465,18 +3113,27 @@
         <v>1590424662</v>
       </c>
       <c r="D72" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E72" s="3" t="n">
         <v>550066654</v>
       </c>
-      <c r="E72" s="3" t="n">
+      <c r="F72" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="G72" s="3" t="n">
         <v>1086436189</v>
       </c>
-      <c r="F72" s="3" t="n">
+      <c r="H72" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="I72" s="3" t="n">
         <v>1636502843</v>
       </c>
-      <c r="G72" s="3" t="n">
+      <c r="J72" s="3" t="n">
         <v>46078181</v>
       </c>
-      <c r="H72" s="4" t="n">
+      <c r="K72" s="4" t="n">
         <v>102.8972250054307</v>
       </c>
     </row>
@@ -2493,18 +3150,27 @@
         <v>1541262682</v>
       </c>
       <c r="D73" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="E73" s="3" t="n">
         <v>650951589</v>
       </c>
-      <c r="E73" s="3" t="n">
+      <c r="F73" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="G73" s="3" t="n">
         <v>870983319</v>
       </c>
-      <c r="F73" s="3" t="n">
+      <c r="H73" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="I73" s="3" t="n">
         <v>1521934908</v>
       </c>
-      <c r="G73" s="3" t="n">
+      <c r="J73" s="3" t="n">
         <v>-19327774</v>
       </c>
-      <c r="H73" s="4" t="n">
+      <c r="K73" s="4" t="n">
         <v>98.74597794225969</v>
       </c>
     </row>
@@ -2521,18 +3187,27 @@
         <v>1340783039</v>
       </c>
       <c r="D74" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E74" s="3" t="n">
         <v>431133242</v>
       </c>
-      <c r="E74" s="3" t="n">
+      <c r="F74" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="G74" s="3" t="n">
         <v>856159167</v>
       </c>
-      <c r="F74" s="3" t="n">
+      <c r="H74" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="I74" s="3" t="n">
         <v>1287292409</v>
       </c>
-      <c r="G74" s="3" t="n">
+      <c r="J74" s="3" t="n">
         <v>-53490630</v>
       </c>
-      <c r="H74" s="4" t="n">
+      <c r="K74" s="4" t="n">
         <v>96.01049323834712</v>
       </c>
     </row>
@@ -2560,7 +3235,16 @@
       <c r="G75" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H75" s="4" t="n">
+      <c r="H75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2588,7 +3272,16 @@
       <c r="G76" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H76" s="4" t="n">
+      <c r="H76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2605,18 +3298,27 @@
         <v>152839375774</v>
       </c>
       <c r="D77" s="3" t="n">
+        <v>171</v>
+      </c>
+      <c r="E77" s="3" t="n">
         <v>152943986565</v>
       </c>
-      <c r="E77" s="3" t="n">
+      <c r="F77" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G77" s="3" t="n">
         <v>74283751435</v>
       </c>
-      <c r="F77" s="3" t="n">
+      <c r="H77" s="3" t="n">
+        <v>180</v>
+      </c>
+      <c r="I77" s="3" t="n">
         <v>227227738000</v>
       </c>
-      <c r="G77" s="3" t="n">
+      <c r="J77" s="3" t="n">
         <v>74388362226</v>
       </c>
-      <c r="H77" s="4" t="n">
+      <c r="K77" s="4" t="n">
         <v>148.6709408810962</v>
       </c>
     </row>
@@ -2633,18 +3335,27 @@
         <v>7278481441</v>
       </c>
       <c r="D78" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="E78" s="3" t="n">
         <v>2279704309</v>
       </c>
-      <c r="E78" s="3" t="n">
+      <c r="F78" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="G78" s="3" t="n">
         <v>5585152500</v>
       </c>
-      <c r="F78" s="3" t="n">
+      <c r="H78" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="I78" s="3" t="n">
         <v>7864856809</v>
       </c>
-      <c r="G78" s="3" t="n">
+      <c r="J78" s="3" t="n">
         <v>586375368</v>
       </c>
-      <c r="H78" s="4" t="n">
+      <c r="K78" s="4" t="n">
         <v>108.0562871905797</v>
       </c>
     </row>
@@ -2661,18 +3372,27 @@
         <v>22848633910</v>
       </c>
       <c r="D79" s="3" t="n">
+        <v>178</v>
+      </c>
+      <c r="E79" s="3" t="n">
         <v>11374715485</v>
       </c>
-      <c r="E79" s="3" t="n">
+      <c r="F79" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="G79" s="3" t="n">
         <v>18278810373</v>
       </c>
-      <c r="F79" s="3" t="n">
+      <c r="H79" s="3" t="n">
+        <v>238</v>
+      </c>
+      <c r="I79" s="3" t="n">
         <v>29653525858</v>
       </c>
-      <c r="G79" s="3" t="n">
+      <c r="J79" s="3" t="n">
         <v>6804891948</v>
       </c>
-      <c r="H79" s="4" t="n">
+      <c r="K79" s="4" t="n">
         <v>129.7824892936893</v>
       </c>
     </row>
@@ -2689,18 +3409,27 @@
         <v>25099404705</v>
       </c>
       <c r="D80" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="E80" s="3" t="n">
         <v>29721544874</v>
       </c>
-      <c r="E80" s="3" t="n">
+      <c r="F80" s="3" t="n">
+        <v>153</v>
+      </c>
+      <c r="G80" s="3" t="n">
         <v>12596295899</v>
       </c>
-      <c r="F80" s="3" t="n">
+      <c r="H80" s="3" t="n">
+        <v>503</v>
+      </c>
+      <c r="I80" s="3" t="n">
         <v>42317840773</v>
       </c>
-      <c r="G80" s="3" t="n">
+      <c r="J80" s="3" t="n">
         <v>17218436068</v>
       </c>
-      <c r="H80" s="4" t="n">
+      <c r="K80" s="4" t="n">
         <v>168.6009738891136</v>
       </c>
     </row>
@@ -2728,7 +3457,16 @@
       <c r="G81" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H81" s="4" t="n">
+      <c r="H81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>